<commit_message>
Update group submission files
</commit_message>
<xml_diff>
--- a/5anhemsiunhan_CS12.xlsx
+++ b/5anhemsiunhan_CS12.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="14000" activeTab="5"/>
+    <workbookView windowWidth="29100" windowHeight="14000" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="0_Hướng dẫn" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="656">
   <si>
     <t>CS12 · Đánh giá sản phẩm AI · Bài tập buổi sáng 16/10/2026</t>
   </si>
@@ -1399,6 +1399,9 @@
   </si>
   <si>
     <t>Tên nhóm và thành viên:</t>
+  </si>
+  <si>
+    <t>Nhóm ___ · Đinh Thị Minh Tâm, Bùi Thị Ngọc Trân, Nguyễn Khánh Linh, Ngô Lê Thuỷ Tiên, Phạm Thành Đạt</t>
   </si>
   <si>
     <t>X1 · Đơn vị công việc AI (4 phút · 1 điểm)</t>
@@ -3658,12 +3661,12 @@
   <sheetData>
     <row r="1" ht="17.35" customHeight="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>12</v>
@@ -3672,7 +3675,7 @@
         <v>234</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:4">
@@ -3752,15 +3755,15 @@
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:4">
       <c r="A10" s="7" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:4">
       <c r="A11" s="3" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="C11" s="8" t="str">
         <f>Xưởng!G7</f>
@@ -3769,10 +3772,10 @@
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:4">
       <c r="A12" s="3" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="C12" s="8" t="str">
         <f>Xưởng!D20</f>
@@ -3781,10 +3784,10 @@
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:4">
       <c r="A13" s="3" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="C13" s="8" t="str">
         <f>Xưởng!C36</f>
@@ -3793,25 +3796,25 @@
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:4">
       <c r="A14" s="3" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C14" s="5">
         <f>COUNTIF(Xưởng!F56:G58,"Đúng")</f>
         <v>6</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:4">
       <c r="A15" s="3" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="C15" s="8" t="str">
         <f>Xưởng!C67</f>
@@ -3820,32 +3823,32 @@
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:4">
       <c r="A16" s="3" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C16" s="5">
         <f>COUNTIF(Xưởng!G72:G84,"Đúng")</f>
         <v>5</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:4">
       <c r="A17" s="3" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C17" s="5">
         <f>COUNTIF(Xưởng!D105:D112,"Đúng")</f>
         <v>4</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
     </row>
   </sheetData>
@@ -3875,10 +3878,10 @@
         <v>322</v>
       </c>
       <c r="C1" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="D1" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="E1" t="s">
         <v>262</v>
@@ -3896,7 +3899,7 @@
         <v>378</v>
       </c>
       <c r="J1" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="K1" t="s">
         <v>395</v>
@@ -3943,10 +3946,10 @@
         <v>391</v>
       </c>
       <c r="K2" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="L2" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="M2" t="s">
         <v>440</v>
@@ -3957,13 +3960,13 @@
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:14">
       <c r="B3" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C3" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="D3" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="E3" t="s">
         <v>271</v>
@@ -3981,10 +3984,10 @@
         <v>385</v>
       </c>
       <c r="J3" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="K3" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="N3" t="s">
         <v>374</v>
@@ -3995,7 +3998,7 @@
         <v>110</v>
       </c>
       <c r="N4" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:14">
@@ -6789,7 +6792,9 @@
         <v>453</v>
       </c>
       <c r="B3" s="14"/>
-      <c r="C3" s="15"/>
+      <c r="C3" s="15" t="s">
+        <v>454</v>
+      </c>
       <c r="D3" s="16"/>
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
@@ -6797,21 +6802,21 @@
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:7">
       <c r="A5" s="7" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:7">
       <c r="A6" s="18" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="7" ht="61.5" customHeight="1" spans="1:7">
       <c r="A7" s="3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B7" s="14"/>
       <c r="C7" s="15" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
@@ -6823,26 +6828,26 @@
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:7">
       <c r="A9" s="7" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:7">
       <c r="A10" s="18" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:7">
       <c r="A11" s="2" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E11" s="20"/>
       <c r="F11" s="20"/>
@@ -6853,13 +6858,13 @@
         <v>90</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C12" s="21">
         <v>3</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
@@ -6870,13 +6875,13 @@
         <v>93</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C13" s="21">
         <v>3</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
@@ -6887,13 +6892,13 @@
         <v>96</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C14" s="21">
         <v>3</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
@@ -6901,7 +6906,7 @@
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:7">
       <c r="A15" s="3" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B15" s="14"/>
       <c r="C15" s="5">
@@ -6911,7 +6916,7 @@
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:7">
       <c r="A16" s="3" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="21">
@@ -6920,7 +6925,7 @@
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:5">
       <c r="A17" s="3" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="5">
@@ -6930,7 +6935,7 @@
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:5">
       <c r="A18" s="3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B18" s="14"/>
       <c r="C18" s="21">
@@ -6943,7 +6948,7 @@
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:5">
       <c r="A19" s="3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B19" s="14"/>
       <c r="C19" s="21">
@@ -6952,7 +6957,7 @@
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:5">
       <c r="A20" s="3" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B20" s="14"/>
       <c r="C20" s="22">
@@ -6966,27 +6971,27 @@
     </row>
     <row r="22" ht="18" customHeight="1" spans="1:5">
       <c r="A22" s="7" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" spans="1:5">
       <c r="A23" s="18" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:5">
       <c r="A24" s="2" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="D24" s="14"/>
       <c r="E24" s="2" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="25" ht="48" customHeight="1" spans="1:5">
@@ -6994,10 +6999,10 @@
         <v>90</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="D25" s="17"/>
       <c r="E25" s="15" t="s">
@@ -7009,10 +7014,10 @@
         <v>93</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D26" s="17"/>
       <c r="E26" s="15" t="s">
@@ -7024,10 +7029,10 @@
         <v>96</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="D27" s="17"/>
       <c r="E27" s="15" t="s">
@@ -7039,10 +7044,10 @@
         <v>109</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="D28" s="17"/>
       <c r="E28" s="15" t="s">
@@ -7054,10 +7059,10 @@
         <v>112</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="D29" s="17"/>
       <c r="E29" s="15" t="s">
@@ -7069,10 +7074,10 @@
         <v>128</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D30" s="17"/>
       <c r="E30" s="15" t="s">
@@ -7084,10 +7089,10 @@
         <v>131</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="D31" s="17"/>
       <c r="E31" s="15" t="s">
@@ -7099,10 +7104,10 @@
         <v>134</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="D32" s="17"/>
       <c r="E32" s="15" t="s">
@@ -7111,7 +7116,7 @@
     </row>
     <row r="33" ht="18" customHeight="1" spans="1:7">
       <c r="B33" s="3" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C33" s="5">
         <f>COUNTIF(E25:E32,"Đại diện")</f>
@@ -7120,7 +7125,7 @@
     </row>
     <row r="34" ht="18" customHeight="1" spans="1:7">
       <c r="B34" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="C34" s="5">
         <f>COUNTIF(E25:E32,"Thử thách")</f>
@@ -7129,7 +7134,7 @@
     </row>
     <row r="35" ht="18" customHeight="1" spans="1:7">
       <c r="B35" s="3" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C35" s="5">
         <f>COUNTIF(E25:E32,"Hồi quy nghiêm trọng")</f>
@@ -7147,12 +7152,12 @@
     </row>
     <row r="38" ht="18" customHeight="1" spans="1:7">
       <c r="A38" s="7" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1" spans="1:7">
       <c r="A39" s="18" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1" spans="1:7">
@@ -7170,10 +7175,10 @@
     </row>
     <row r="41" ht="18" customHeight="1" spans="1:7">
       <c r="A41" s="3" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C41" s="20"/>
       <c r="D41" s="20"/>
@@ -7195,7 +7200,7 @@
     <row r="43" ht="18" customHeight="1" spans="1:7">
       <c r="A43" s="3"/>
       <c r="B43" s="4" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="C43" s="20"/>
       <c r="D43" s="20"/>
@@ -7206,7 +7211,7 @@
     <row r="44" ht="18" customHeight="1" spans="1:7">
       <c r="A44" s="3"/>
       <c r="B44" s="4" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="C44" s="20"/>
       <c r="D44" s="20"/>
@@ -7216,10 +7221,10 @@
     </row>
     <row r="45" ht="18" customHeight="1" spans="1:7">
       <c r="A45" s="3" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C45" s="20"/>
       <c r="D45" s="20"/>
@@ -7241,7 +7246,7 @@
     <row r="47" ht="18" customHeight="1" spans="1:7">
       <c r="A47" s="3"/>
       <c r="B47" s="4" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="C47" s="20"/>
       <c r="D47" s="20"/>
@@ -7252,7 +7257,7 @@
     <row r="48" ht="18" customHeight="1" spans="1:7">
       <c r="A48" s="3"/>
       <c r="B48" s="4" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C48" s="20"/>
       <c r="D48" s="20"/>
@@ -7263,7 +7268,7 @@
     <row r="49" ht="18" customHeight="1" spans="1:7">
       <c r="A49" s="3"/>
       <c r="B49" s="4" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C49" s="20"/>
       <c r="D49" s="20"/>
@@ -7273,10 +7278,10 @@
     </row>
     <row r="50" ht="18" customHeight="1" spans="1:7">
       <c r="A50" s="3" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C50" s="20"/>
       <c r="D50" s="20"/>
@@ -7298,7 +7303,7 @@
     <row r="52" ht="18" customHeight="1" spans="1:7">
       <c r="A52" s="3"/>
       <c r="B52" s="4" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="C52" s="20"/>
       <c r="D52" s="20"/>
@@ -7309,7 +7314,7 @@
     <row r="53" ht="18" customHeight="1" spans="1:7">
       <c r="A53" s="3"/>
       <c r="B53" s="4" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C53" s="20"/>
       <c r="D53" s="20"/>
@@ -7322,25 +7327,25 @@
         <v>278</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E55" s="14"/>
       <c r="F55" s="2" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="56" ht="61.5" customHeight="1" spans="1:7">
       <c r="A56" s="3" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B56" s="21">
         <v>3</v>
@@ -7349,7 +7354,7 @@
         <v>105</v>
       </c>
       <c r="D56" s="15" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="E56" s="17"/>
       <c r="F56" s="19" t="str">
@@ -7363,7 +7368,7 @@
     </row>
     <row r="57" ht="61.5" customHeight="1" spans="1:7">
       <c r="A57" s="3" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B57" s="21">
         <v>2</v>
@@ -7372,7 +7377,7 @@
         <v>103</v>
       </c>
       <c r="D57" s="15" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="E57" s="17"/>
       <c r="F57" s="19" t="str">
@@ -7386,7 +7391,7 @@
     </row>
     <row r="58" ht="61.5" customHeight="1" spans="1:7">
       <c r="A58" s="3" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B58" s="21">
         <v>4</v>
@@ -7395,7 +7400,7 @@
         <v>110</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E58" s="17"/>
       <c r="F58" s="19" t="str">
@@ -7409,127 +7414,127 @@
     </row>
     <row r="60" ht="18" customHeight="1" spans="1:7">
       <c r="A60" s="7" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1" spans="1:7">
       <c r="A61" s="18" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1" spans="1:7">
       <c r="A62" s="2" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
     </row>
     <row r="63" ht="78" customHeight="1" spans="1:7">
       <c r="A63" s="3" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B63" s="15" t="s">
         <v>77</v>
       </c>
       <c r="C63" s="15" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="D63" s="15" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="E63" s="15" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F63" s="15" t="s">
         <v>359</v>
       </c>
       <c r="G63" s="15" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
     <row r="64" ht="78" customHeight="1" spans="1:7">
       <c r="A64" s="3" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B64" s="15" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C64" s="15" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="D64" s="15" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="E64" s="15" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F64" s="15" t="s">
         <v>359</v>
       </c>
       <c r="G64" s="15" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
     </row>
     <row r="65" ht="78" customHeight="1" spans="1:7">
       <c r="A65" s="3" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="C65" s="15" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="D65" s="15" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="E65" s="15" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="F65" s="15" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="G65" s="15" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="66" ht="78" customHeight="1" spans="1:7">
       <c r="A66" s="3" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C66" s="15" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="D66" s="15" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="E66" s="15" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="F66" s="15" t="s">
         <v>371</v>
       </c>
       <c r="G66" s="15" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
     </row>
     <row r="67" ht="33" customHeight="1" spans="1:7">
@@ -7541,17 +7546,17 @@
         <v>Đạt</v>
       </c>
       <c r="D67" s="23" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="69" ht="18" customHeight="1" spans="1:7">
       <c r="A69" s="7" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="70" ht="18" customHeight="1" spans="1:7">
       <c r="A70" s="18" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="71" ht="18" customHeight="1" spans="1:7">
@@ -7559,17 +7564,17 @@
         <v>401</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>371</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="E71" s="14"/>
       <c r="F71" s="2" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="G71" s="2" t="s">
         <v>210</v>
@@ -7586,7 +7591,7 @@
         <v>403</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="E72" s="14"/>
       <c r="F72" s="21">
@@ -7608,7 +7613,7 @@
         <v>404</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="E73" s="14"/>
       <c r="F73" s="21">
@@ -7630,7 +7635,7 @@
         <v>403</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="E74" s="14"/>
       <c r="F74" s="21">
@@ -7652,7 +7657,7 @@
         <v>404</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="E75" s="14"/>
       <c r="F75" s="21">
@@ -7674,7 +7679,7 @@
         <v>403</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="E76" s="14"/>
       <c r="F76" s="24">
@@ -7697,7 +7702,7 @@
         <v>403</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="E77" s="14"/>
       <c r="F77" s="24">
@@ -7720,7 +7725,7 @@
         <v>404</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="E78" s="14"/>
       <c r="F78" s="25">
@@ -7738,7 +7743,7 @@
         <v>403</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="E79" s="14"/>
       <c r="F79" s="5">
@@ -7768,7 +7773,7 @@
         <v>404</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="E81" s="20"/>
       <c r="F81" s="20"/>
@@ -7785,7 +7790,7 @@
         <v>403</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="E82" s="20"/>
       <c r="F82" s="20"/>
@@ -7802,7 +7807,7 @@
         <v>404</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="E83" s="20"/>
       <c r="F83" s="20"/>
@@ -7819,7 +7824,7 @@
         <v>403</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="E84" s="14"/>
       <c r="F84" s="15" t="s">
@@ -7909,12 +7914,12 @@
     </row>
     <row r="94" ht="18" customHeight="1" spans="1:7">
       <c r="A94" s="7" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="95" ht="18" customHeight="1" spans="1:7">
       <c r="A95" s="18" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
     </row>
     <row r="96" ht="18" customHeight="1" spans="1:7">
@@ -7923,10 +7928,10 @@
       </c>
       <c r="B96" s="14"/>
       <c r="C96" s="2" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>330</v>
@@ -7950,25 +7955,25 @@
         <v>334</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="98" ht="18" customHeight="1" spans="1:7">
       <c r="A98" s="4" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B98" s="14"/>
       <c r="C98" s="4" t="s">
         <v>359</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="99" ht="18" customHeight="1" spans="1:7">
@@ -7980,13 +7985,13 @@
         <v>359</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="100" ht="18" customHeight="1" spans="1:7">
@@ -7995,34 +8000,34 @@
       </c>
       <c r="B100" s="14"/>
       <c r="C100" s="4" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="E100" s="4" t="s">
         <v>344</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
     </row>
     <row r="101" ht="18" customHeight="1" spans="1:7">
       <c r="A101" s="4" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B101" s="14"/>
       <c r="C101" s="4" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="D101" s="4" t="s">
         <v>333</v>
       </c>
       <c r="E101" s="4" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
     </row>
     <row r="102" ht="18" customHeight="1" spans="1:7">
@@ -8040,21 +8045,21 @@
         <v>340</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
     <row r="103" ht="18" customHeight="1" spans="1:7">
       <c r="A103" s="23" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
     </row>
     <row r="105" ht="18" customHeight="1" spans="1:7">
       <c r="A105" s="3" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B105" s="14"/>
       <c r="C105" s="15" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="D105" s="19" t="str">
         <f>IF(C105="","",IF(C105="Phát hành","Đúng","Chưa đúng"))</f>
@@ -8063,11 +8068,11 @@
     </row>
     <row r="106" ht="78" customHeight="1" spans="1:7">
       <c r="A106" s="3" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B106" s="14"/>
       <c r="C106" s="15" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="D106" s="16"/>
       <c r="E106" s="16"/>
@@ -8076,17 +8081,17 @@
     </row>
     <row r="107" ht="18" customHeight="1" spans="1:7">
       <c r="C107" s="23" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
     </row>
     <row r="109" ht="18" customHeight="1" spans="1:7">
       <c r="A109" s="18" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
     </row>
     <row r="110" ht="18" customHeight="1" spans="1:7">
       <c r="A110" s="3" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B110" s="14"/>
       <c r="C110" s="26">
@@ -8099,7 +8104,7 @@
     </row>
     <row r="111" ht="18" customHeight="1" spans="1:7">
       <c r="A111" s="3" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="B111" s="14"/>
       <c r="C111" s="21">
@@ -8112,7 +8117,7 @@
     </row>
     <row r="112" ht="33" customHeight="1" spans="1:7">
       <c r="A112" s="3" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B112" s="14"/>
       <c r="C112" s="26">
@@ -8254,157 +8259,157 @@
   <sheetData>
     <row r="1" ht="17.35" customHeight="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:6">
       <c r="A2" s="9" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:6">
       <c r="A4" s="2" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
     </row>
     <row r="5" ht="33" customHeight="1" spans="1:6">
       <c r="A5" s="3" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B5" s="10">
         <v>1</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="F5" s="11"/>
     </row>
     <row r="6" ht="33" customHeight="1" spans="1:6">
       <c r="A6" s="3" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B6" s="10">
         <v>1</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="F6" s="11"/>
     </row>
     <row r="7" ht="33" customHeight="1" spans="1:6">
       <c r="A7" s="3" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B7" s="10">
         <v>2</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="F7" s="11"/>
     </row>
     <row r="8" ht="33" customHeight="1" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B8" s="10">
         <v>1.5</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="F8" s="11"/>
     </row>
     <row r="9" ht="48" customHeight="1" spans="1:6">
       <c r="A9" s="3" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B9" s="10">
         <v>2</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="F9" s="11"/>
     </row>
     <row r="10" ht="33" customHeight="1" spans="1:6">
       <c r="A10" s="3" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B10" s="10">
         <v>1</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="F10" s="11"/>
     </row>
     <row r="11" ht="48" customHeight="1" spans="1:6">
       <c r="A11" s="3" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B11" s="10">
         <v>1.5</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="F11" s="11"/>
     </row>

</xml_diff>